<commit_message>
2026.10.19/김나은/문서 React+Django API 기준으로 정리, Cognito→자체 회원·세션 로그인, django-htmx 제거
</commit_message>
<xml_diff>
--- a/산출물/01_기획/4팀_요구사항정의서.xlsx
+++ b/산출물/01_기획/4팀_요구사항정의서.xlsx
@@ -865,7 +865,7 @@
       <c r="F10" s="14" t="inlineStr">
         <is>
           <t>입력: 금융기관 인증·추가인증 결과, 조회 동의와 내부 연결 요청 ID를 사용한다.
-처리·저장: API 제공 서비스는 CODEF로 정하고 은행·카드 조회에 적용한다. CODEF API 호출 인증, 금융기관 계정 연결, 앱 Cognito 로그인은 구분한다. 연결 상태·동의 범위·시각을 기록한다.
+처리·저장: API 제공 서비스는 CODEF로 정하고 은행·카드 조회에 적용한다. CODEF API 호출 인증, 금융기관 계정 연결, 앱 로그인(Django 자체 회원)은 구분한다. 연결 상태·동의 범위·시각을 기록한다.
 예외: 취소·인증 실패·동의 철회·지연은 각각 안내하고 성공 상태를 만들지 않는다.
 검수: 동의 없는 조회와 재시도 중복 연결을 차단한다. 데모·테스트·운영 환경을 구분하며 지원 기관·이용 계약·운영 접근 권한은 별도 검증한다.
 참고 반영(ACC-005): 연결 요청 ID를 인증 사용자·기관·동의 버전·만료 시각에 묶는다. 추가인증의 후속 요청은 동일 사용자·연결 흐름인지 검사하고 만료·재사용·타인 요청을 거부한다. CODEF 실제 인증 절차에서 검증하며 금융결제원 콜백·토큰 교환 방식을 전제하지 않는다.
@@ -2357,7 +2357,7 @@
       <c r="F53" s="17" t="inlineStr">
         <is>
           <t>입력: 제안 식별값, 기준 예산 버전, 명시적 승인과 중복 요청 식별 정보를 받는다.
-처리·저장/예외: API에서 JWT 인증·소유권을 검증하고 최신 자료로 다시 계산한다. 금액·영향 변경 시 재승인을 요청하며, 예산 버전 비교·멱등성 검사·변경 기록 저장을 원자적으로 처리한다. 비동기 작업자와 메시지 재처리는 제안 생성까지만 수행한다.
+처리·저장/예외: API에서 로그인 세션·소유권을 검증하고 최신 자료로 다시 계산한다. 금액·영향 변경 시 재승인을 요청하며, 예산 버전 비교·멱등성 검사·변경 기록 저장을 원자적으로 처리한다. 비동기 작업자와 메시지 재처리는 제안 생성까지만 수행한다.
 잔소리: 이번 달 예산 조정 3회째부터 반복 조정 안내 문구(잔소리)를 보여준다. 안내만 하며 조정을 막지 않는다. 자물쇠 변경 잔소리는 BUD-012를 따른다.
 검수기준: 무승인·타인 요청·버전 충돌은 적용되지 않고 동시·재시도 요청은 한 번만 반영되며, 변경 전후 금액·승인 시각·요청 주체·근거 버전을 조회할 수 있어야 한다.</t>
         </is>
@@ -3356,7 +3356,7 @@
       <c r="E81" s="17" t="inlineStr">
         <is>
           <t>주요 화면·공통 승인 흐름
-Django 템플릿·HTMX 기반 모바일 웹에 회원가입·로그인·온보딩·홈·거래·예산 조정·통합 챗봇·소비 분석 화면(2차)·마이 화면을 제공하고 여러 진입점에서 같은 예산 조정·승인 흐름으로 이동하게 한다. 통합 챗봇은 하단 탭(기존 마이 자리)에 둔다.</t>
+React 기반 모바일 웹(데이터는 Django API)에 회원가입·로그인·온보딩·홈·거래·예산 조정·통합 챗봇·소비 분석 화면(2차)·마이 화면을 제공하고 여러 진입점에서 같은 예산 조정·승인 흐름으로 이동하게 한다. 통합 챗봇은 하단 탭(기존 마이 자리)에 둔다.</t>
         </is>
       </c>
       <c r="F81" s="17" t="inlineStr">
@@ -3436,7 +3436,7 @@
           <t>요청 분배와 비동기 작업
 대상·상황
 사용자가 조회 또는 에이전트 처리가 필요한 요청을 한다.
-처리·출력: API는 JWT·소유권을 검사하고 일반 조회는 DB/계산 엔진으로 즉시 처리한다. 라우터(AGT-001)가 지정한 에이전트 작업만 작업 ID를 반환하고 Worker가 수행한다.</t>
+처리·출력: API는 로그인 세션·소유권을 검사하고 일반 조회는 DB/계산 엔진으로 즉시 처리한다. 라우터(AGT-001)가 지정한 에이전트 작업만 작업 ID를 반환하고 Worker가 수행한다.</t>
         </is>
       </c>
       <c r="F83" s="14" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>구현안: 모바일 웹(Django)의 Cognito 로그인, API의 JWT 서명·issuer·audience/client·token_use·만료 검증은 Cognito Access Token 규격에 맞추고 JWKS로 서명을 검증한다. 개인 RDS는 외부 공개하지 않고 서버 역할별 최소 권한을 둔다. CODEF client secret·API 토큰은 백엔드에서만 관리하고 웹·LLM에 전달하지 않는다. 실제 키 발급·등록은 별도 작업이다.
+          <t>구현안: Django 자체 회원과 세션 로그인을 쓴다. 세션 쿠키는 HttpOnly·Secure·SameSite로 설정하고, 상태를 바꾸는 요청은 CSRF 토큰을 검증하며, 비밀번호는 Django 기본 해시로만 저장한다. 개인 RDS는 외부 공개하지 않고 서버 역할별 최소 권한을 둔다. CODEF client secret·API 토큰은 백엔드에서만 관리하고 웹·LLM에 전달하지 않는다. 실제 키 발급·등록은 별도 작업이다.
 예외: 만료·변조·타인 ID 요청은 거부한다. 토큰·계좌번호·거래 원문·비밀값을 로그에 남기지 않는다.
 검수 기준: 사용자 A가 B의 거래·job·proposal을 읽거나 적용할 수 없음, 로그 비밀값 검사, Worker의 승인 예산 쓰기 거부.
 진입 권한: 서버도 연결·동의·최초 잔액 성공을 검사해 화면 우회를 차단한다. 미연결 상태의 가입·로그인·복구·연결·도움말 접근은 허용한다.</t>
@@ -4897,7 +4897,7 @@
       <c r="E124" s="11" t="inlineStr">
         <is>
           <t>실행 구조와 쓰기 권한(구현안)
-Django 모바일 웹(템플릿·HTMX), Cognito 인증, AWS EC2 한 대의 Docker Compose TLS Reverse Proxy/Django/AI Worker 3개 컨테이너, 관리형 SQS·비공개 RDS PostgreSQL·S3 모델 저장·CloudWatch 구성을 기준으로 상세 설계한다. 네이티브 앱은 후속이다.</t>
+React 모바일 웹 + Django API(DRF), Django 세션 인증, AWS EC2 한 대의 Docker Compose TLS Reverse Proxy/Django/AI Worker 3개 컨테이너, 관리형 SQS·비공개 RDS PostgreSQL·S3 모델 저장·CloudWatch 구성을 기준으로 상세 설계한다. 네이티브 앱은 후속이다.</t>
         </is>
       </c>
       <c r="F124" s="11" t="inlineStr">
@@ -5243,7 +5243,7 @@
       <c r="F131" s="14" t="inlineStr">
         <is>
           <t>입력: 이메일·비밀번호·필수/선택 약관 버전과 동의값.
-처리·저장: Cognito 계정을 생성하고 내부 사용자 식별값·필수 동의 버전을 연결한다. 비밀번호 해시 처리는 Cognito가 담당하며 앱 DB에 비밀번호를 저장하지 않는다.
+처리·저장: 앱 DB(app_user)에 계정을 생성하고 필수 동의 버전을 연결한다. 비밀번호는 Django 기본 해시로만 저장하고 원문은 저장·로그하지 않는다.
 예외: 중복 이메일·정책 위반·필수 동의 누락은 가입 완료로 처리하지 않는다. 선택 동의 거절은 가입을 막지 않는다.
 검수: 정상 가입 후 계정이 생성되고 잘못된 입력은 거절된다.
 흐름: 가입은 금융기관 연결 전 가능하다. 가입 성공 후 필수 계좌 연결·동의·최초 잔액 조회로 안내하며 핵심 예산 진입 완료와 구분한다.</t>
@@ -5281,9 +5281,9 @@
       </c>
       <c r="F132" s="14" t="inlineStr">
         <is>
-          <t>입력: 이메일·비밀번호 또는 유효한 Cognito 세션.
-처리·저장: 인증 성공 후 만료 있는 토큰으로 API에 접근하며 로그아웃·비밀번호 변경·계정 해제 시 세션 폐기 상태를 서버에도 반영한다.
-예외: 실패 문구로 계정 존재를 드러내지 않는다. 이미 발급된 JWT의 잔여 유효성도 고려해 폐기 이후 요청을 차단하는 검증을 둔다.
+          <t>입력: 이메일·비밀번호 또는 유효한 로그인 세션.
+처리·저장: 인증 성공 후 만료 있는 세션으로 API에 접근하며 로그아웃·비밀번호 변경·계정 해제 시 세션 폐기 상태를 서버에도 반영한다.
+예외: 실패 문구로 계정 존재를 드러내지 않는다. 서버 세션을 삭제해 폐기 이후 요청을 차단한다.
 검수: 로그인 시 세션이 생성되고 로그아웃 시 종료된다.
 진입 분기: 로그인 후 계좌 연결 상태를 확인한다. 미연결·최초 잔액 조회 미완료는 연결/재시도 화면으로, 완료 상태는 권한·최신성 검사를 거쳐 홈으로 이동한다.</t>
         </is>
@@ -5316,8 +5316,8 @@
       </c>
       <c r="F133" s="14" t="inlineStr">
         <is>
-          <t>입력: 이메일 확인과 Cognito 복구 코드·새 비밀번호.
-처리·저장: Cognito의 재설정 흐름에서 유효시간·일회 사용을 검증한다. 완료·새 요청 이후 이전 코드와 기존 세션의 처리 규칙을 검증하고 이력에는 비밀값을 남기지 않는다.
+          <t>입력: 이메일 확인과 복구 링크(일회용 토큰)·새 비밀번호.
+처리·저장: Django 비밀번호 재설정 흐름에서 유효시간·일회 사용을 검증한다. 완료·새 요청 이후 이전 코드와 기존 세션의 처리 규칙을 검증하고 이력에는 비밀값을 남기지 않는다.
 예외: 만료·재사용·틀린 코드는 거절하고 새 요청 경로를 안내한다. 확인되지 않은 계정의 비밀번호를 변경하지 않는다.
 검수: 만료·재사용 요청은 거절되고 새 비밀번호로 로그인할 수 있다.</t>
         </is>

</xml_diff>

<commit_message>
2026.10.21/김나은/고정지출 C-05~C-14 결정 반영·category_detail 삭제·created_at 추가·요청 번호(idempotency_record)·주소 404 JSON·결정기록
</commit_message>
<xml_diff>
--- a/산출물/01_기획/4팀_요구사항정의서.xlsx
+++ b/산출물/01_기획/4팀_요구사항정의서.xlsx
@@ -586,7 +586,7 @@
     <row r="2" ht="25.5" customHeight="1" s="18">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21 | 카테고리 최소 금액(온보딩 선택 입력) 반영 | 카테고리 10개 기준·우선순위 4위부터 선택 반영 | LLM 라우터(자연어 요청 분석) 반영 | 기획서 MVP 재정의 반영(총 146개) | 챗봇 소비 분석 답변을 템플릿 문장으로 확정(CHT-006·RPT-001·RPT-004·AGT-001) | 고정지출 범위·대출 상환·저축 감지 반영(TXN-005·008·BUD-001·003) | 날짜 보정 규칙(말일)·고정지출 금액·출금일 범위 확정(BUD-004·TXN-008) | 고정지출 주기·상태·감지 조건·온보딩 후 추가 반영(TXN-008·BUD-005·011) | 우선순위: 1차(MVP) 89 · 2차 12 · 3차 12 · 후순위 25 (카드 OCR은 검증 필요, 별도 ID 없음) | 복지·대출은 비교 정보만 | 입력·처리·출력·예외·검수 상세화</t>
+          <t>2026-10-21 | 카테고리 최소 금액(온보딩 선택 입력) 반영 | 카테고리 10개 기준·우선순위 4위부터 선택 반영 | LLM 라우터(자연어 요청 분석) 반영 | 기획서 MVP 재정의 반영(총 146개) | 챗봇 소비 분석 답변을 템플릿 문장으로 확정(CHT-006·RPT-001·RPT-004·AGT-001) | 고정지출 범위·대출 상환·저축 감지 반영(TXN-005·008·BUD-001·003) | 날짜 보정 규칙(말일)·고정지출 금액·출금일 범위 확정(BUD-004·TXN-008) | 고정지출 주기·상태·감지 조건·온보딩 후 추가 반영(TXN-008·BUD-005·011) | 고정지출 수정·중지 적용 시점(TXN-008·BUD-005) | 고정지출 목록 구성(TXN-008) | 같은 비용 찾기·카드값 첫 청구서만 예산 차감(COM-004·TXN-008·009·BUD-001) | 에러 fields 규칙·요청 번호로 중복 저장 방지(NFR-003) | 카드 거래↔고정지출 연결·결제 확인(TXN-008) | 우선순위: 1차(MVP) 89 · 2차 12 · 3차 12 · 후순위 25 (카드 OCR은 검증 필요, 별도 ID 없음) | 복지·대출은 비교 정보만 | 입력·처리·출력·예외·검수 상세화</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       <c r="F21" s="17" t="inlineStr">
         <is>
           <t>입력: 확인된 거래 이력과 현재 등록된 고정지출·예정지출 목록을 사용한다.
-처리·저장: 후보의 근거 거래·추정 주기·확인 필요 항목을 저장하고 승인 시 기존 항목과 중복을 검사해 하나의 의무지출로 연결한다. API의 자동이체·반복 출금만으로 모든 향후 지출을 확정하지 않는다. 고정지출은 매달 금액·날짜가 정해져 피할 수 없는 돈이며 매월 주기만 받는다(1년에 한 번 내는 돈은 비정기지출 준비금 BUD-011, 매주·매일 사는 것은 생활비 카테고리 예산). 감지 조건: 같은 받는 곳으로 한 달에 1건만 나가고, 매달 같은 날 ±3일, 같은 금액(변동 청구는 ±10%)이 3달 연속이면 후보로 만든다(시작 값이며 데이터로 조정). 상태: 자동 발견은 후보(suggested) → 사용자가 맞다고 하면 확정(confirmed), 아니라고 하면 무시(ignored, 같은 후보를 다시 묻지 않음), 더 이상 안 나가면 중지(stopped). 직접 추가는 바로 확정. 출처는 직접 등록(manual)·반복 탐지(detected)로 남기고 후보를 고쳐 확정해도 detected를 유지한다. 예산에는 확정만 들어간다. 온보딩이 끝난 뒤 확정된 고정지출의 이번 주기 몫: 결제일이 지났고 맞는 거래가 있으면 그 거래를 생활비에서 고정비로 옮기고, 결제일이 남았으면 결제일에 나갈 돈으로 예약하며, 결제일이 지났는데 거래가 없으면 이번 주기는 건드리지 않는다. 옮기거나 예약한 금액은 여윳돈으로 먼저 메우고 모자라면 예산 조정을 제안한다(사용자 승인 후 반영, BUD-005). 다음 주기부터는 고정비로 먼저 뺀다. 후보를 만들기 전에 먼저 거른다: ① 등록된 대출과 맞는 반복 출금(받는 곳 = 대출 기관, 납부일 ±3일, 금액 ≈ 월 상환 예정액)은 고정지출 후보에서 빼고 그 대출의 상환 완료로 연결한다. 대출 상환으로 보이는데 등록된 대출이 없으면 고정지출 대신 대출 등록(ACC-006)으로 안내하고 감지한 금액·납부일을 미리 채운다. ② 내 계좌끼리의 정기 이체는 고정지출 후보에서 빼고 저축 후보(TXN-005)로 묻는다. 고정지출 금액은 1,000원 ~ 1억 원이고(범위 밖은 저장하지 않음), 출금일은 비워 둘 수 있다(1~31, 비우면 '출금일 확인 필요' 표시). 고정지출 합계가 월급보다 커도 등록은 막지 않고 예산을 만들 때 부족액으로 안내한다(BUD-001). 고정지출 카테고리는 10개 + 기타 중 필수 선택이며(항목 이름으로 미리 골라 둠) 저축·투자·대출 상환·카드값은 고정지출로 받지 않는다.
+처리·저장: 후보의 근거 거래·추정 주기·확인 필요 항목을 저장하고 승인 시 기존 항목과 중복을 검사해 하나의 의무지출로 연결한다. API의 자동이체·반복 출금만으로 모든 향후 지출을 확정하지 않는다. 고정지출은 매달 금액·날짜가 정해져 피할 수 없는 돈이며 매월 주기만 받는다(1년에 한 번 내는 돈은 비정기지출 준비금 BUD-011, 매주·매일 사는 것은 생활비 카테고리 예산). 감지 조건: 같은 받는 곳으로 한 달에 1건만 나가고, 매달 같은 날 ±3일, 같은 금액(변동 청구는 ±10%)이 3달 연속이면 후보로 만든다(시작 값이며 데이터로 조정). 상태: 자동 발견은 후보(suggested) → 사용자가 맞다고 하면 확정(confirmed), 아니라고 하면 무시(ignored, 같은 후보를 다시 묻지 않음), 더 이상 안 나가면 중지(stopped). 직접 추가는 바로 확정. 출처는 직접 등록(manual)·반복 탐지(detected)로 남기고 후보를 고쳐 확정해도 detected를 유지한다. 예산에는 확정만 들어간다. 온보딩이 끝난 뒤 확정된 고정지출의 이번 주기 몫: 결제일이 지났고 맞는 거래가 있으면 그 거래를 생활비에서 고정비로 옮기고, 결제일이 남았으면 결제일에 나갈 돈으로 예약하며, 결제일이 지났는데 거래가 없으면 이번 주기는 건드리지 않는다. 옮기거나 예약한 금액은 여윳돈으로 먼저 메우고 모자라면 예산 조정을 제안한다(사용자 승인 후 반영, BUD-005). 다음 주기부터는 고정비로 먼저 뺀다. 같은 비용 찾기(10/21 확정): 고정지출 이름은 사용자가 붙인 별명이므로 이름으로는 맞추지 않는다. ① 기억해 둔 가맹점(자동 발견 후보의 근거 거래 또는 등록 때 사용자가 고른 거래)이 있으면 그 가맹점 + 같은 카드·계좌 + 금액 ±10%로 연결한다. ② 없으면 같은 카드·계좌 + 금액 ±10% + 날짜 ±3일로 찾아 1건이면 '이 결제가 맞나요?'로 한 번 확인하고(여러 건이면 고르게 함, 0건이면 연결하지 않음), 확인한 가맹점을 기억한다. 연결 근거가 약하면 자동으로 합치지 않는다(TXN-009). 연결하면 그 거래의 충당 재원(spending_allocation)을 고정비(fixed)로 기록해 생활비 카테고리 사용액에서 빼고, 그 거래 ID를 고정지출의 근거 거래(evidence)에 더해 가맹점을 기억한다. 매칭은 거래 분류가 끝난 직후에 돌린다. '이 결제가 맞나요?' 확인은 고정지출 목록 응답의 결제 제안(evidenceSuggestion: 거래·가맹점·날짜·금액, 없으면 null)으로 보여주고, 사용자가 맞다고 하면 고정지출 수정의 근거 거래 지정(evidenceTransactionId)으로 확정한다. 아니라고 하면 따로 저장하지 않고 다음 달 새 결제가 오면 다시 묻는다. 1차에서 '이 결제가 맞나요?' 확인과 근거 거래 지정은 카드로 내는 고정지출에만 있다. 계좌로 내는 고정지출은 출금일의 납부 예정과 실제 출금을 날짜·금액으로 맞추므로 사용자에게 묻지 않는다. 납부 예정은 계좌·결제 수단 모름 항목에 출금일이 있을 때만 만들고, 카드로 바꾸거나 출금일을 비우면 이번 달 미납 납부 예정을 취소한다(카드값과 두 번 빼지 않기 위해). 수정·중지(10/21 확정): 금액을 바꾸면 아직 내지 않은 회차(이번 달 미납분과 앞으로의 회차)의 납부 예정만 새 금액으로 바꾸고 이미 냈거나 일부 낸 회차는 그대로 둔다. 이번 달 미납분의 차액은 늘어나면 여윳돈에서 먼저 메우고(모자라면 예산 조정 제안), 줄어들면 여윳돈으로 돌린다. 중지하면 이번 달 미납분의 납부 예정을 취소해 그 금액을 여윳돈으로 돌리고, 이미 냈으면 다음 달부터 없앤다. 중지한 항목은 기록으로 남기며 1차에서는 다시 시작 대신 새로 추가한다. 이미 중지한 항목을 다시 중지하면 같은 결과이므로 성공으로 답한다. 변경 전 금액은 지난 회차의 납부 예정 기록과 승인된 예산의 계산 입력(input_snapshot)으로 남는다. 승인 전 예산 초안은 바뀐 금액으로 다시 계산하고, 바뀌기 전에 만든 초안은 만료되어 승인할 수 없다(COM-005). 고정지출 화면(10/21 확정): 후보는 '새로 찾았어요' 칸에 먼저(최근에 찾은 순, 맞아요/아니에요), 확정은 '내 고정지출' 칸에 출금일 빠른 순(출금일 모름은 맨 아래)으로 보여준다. 중지·무시는 기본 목록에 없다. 페이지는 나누지 않는다. 합계는 확정 항목의 월 금액 합만 보여주고 후보는 넣지 않는다. 다음 급여일까지 남은 납부액은 홈 계산과 함께 정한다. 후보를 만들기 전에 먼저 거른다: ① 등록된 대출과 맞는 반복 출금(받는 곳 = 대출 기관, 납부일 ±3일, 금액 ≈ 월 상환 예정액)은 고정지출 후보에서 빼고 그 대출의 상환 완료로 연결한다. 대출 상환으로 보이는데 등록된 대출이 없으면 고정지출 대신 대출 등록(ACC-006)으로 안내하고 감지한 금액·납부일을 미리 채운다. ② 내 계좌끼리의 정기 이체는 고정지출 후보에서 빼고 저축 후보(TXN-005)로 묻는다. 고정지출 금액은 1,000원 ~ 1억 원이고(범위 밖은 저장하지 않음), 출금일은 비워 둘 수 있다(1~31, 비우면 '출금일 확인 필요' 표시). 고정지출 합계가 월급보다 커도 등록은 막지 않고 예산을 만들 때 부족액으로 안내한다(BUD-001). 고정지출 카테고리는 10개 + 기타 중 필수 선택이며(항목 이름으로 미리 골라 둠) 저축·투자·대출 상환·카드값은 고정지출로 받지 않는다.
 예외: 일회성 동일금액 거래와 변동 청구는 별도 확인한다.
 검수: 후보 생성만으로 예산이 변하지 않고 같은 후보의 승인 재시도에도 비용은 한 번만 반영되며 실제 납부 후 남은 예약액이 해소된다.
 참고 반영(FIX-001): 구독 후보도 같은 경로로 처리하며 가맹점·금액 범위·반복 주기·다음 결제일 후보·출금 계좌·근거 거래·신뢰도를 저장한다. 미확정 다음 결제일은 확정 의무가 아니다.</t>
@@ -1276,7 +1276,7 @@
       <c r="F22" s="17" t="inlineStr">
         <is>
           <t>입력: 카드 구분, 결제일, 청구기간, 확인 금액과 관련 거래를 받는다.
-처리·저장: 내부 청구 의무 ID와 미납액을 저장하며 소비 실적은 확인된 카드 구매에서 별도로 집계한다. 계좌 납부가 확인되면 잔액 감소와 동시에 해당 예약을 해소하고 새 소비를 만들지 않는다.
+처리·저장: 내부 청구 의무 ID와 미납액을 저장하며 소비 실적은 확인된 카드 구매에서 별도로 집계한다. 카드값을 예산에서 먼저 빼는 것은 서비스 시작 전 사용분이 담긴 첫 청구서만이다(10/21 확정). 그 뒤 청구서는 카드로 긁을 때 이미 생활비·고정비에서 빠진 돈이므로 예산에서 다시 빼지 않고, 꼭 나갈 돈과 실제 계좌 납부의 연결에만 쓴다. 청구서 항목 중 카드로 내는 고정지출과 같은 비용은 연결해 '그중 고정비'로 나눠 보여준다. 계좌 납부가 확인되면 잔액 감소와 동시에 해당 예약을 해소하고 새 소비를 만들지 않는다.
 예외: 연결 근거가 약하면 자동 합산·통합하지 않고 확인 요청을 표시하며 카드 구매 미수집을 소비 0원으로 단정하지 않는다.
 검수: 30만원 청구 등록·부분 납부·전액 납부 각 단계에서 남은 의무만 예약되고 안전 소비액이 이중 감소하지 않는다.
 참고 반영(CARD-004): 수동 확정값과 조회값이 다르면 차이를 보여주고 확인 후 새 계산 초안에 반영한다. 할부 전체 구매액과 현재 회차 납부액을 분리한다.
@@ -1288,7 +1288,11 @@
           <t>1차(MVP)</t>
         </is>
       </c>
-      <c r="H22" s="15" t="n"/>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>10/21 수정</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="206" customHeight="1" s="18">
       <c r="A23" s="28" t="n"/>
@@ -1315,7 +1319,7 @@
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>입력: 확인된 월 실수령액, 고정비(확정 고정지출)·대출 월 상환 예정액(ACC-006)·확정 카드대금·이번 회차 할부금, 저축 금액과 쿠션 조건을 사용한다.
+          <t>입력: 확인된 월 실수령액, 고정비(확정 고정지출)·대출 월 상환 예정액(ACC-006)·확정 카드대금(서비스 시작 전 사용분이 담긴 첫 청구서만, TXN-009)·이번 회차 할부금, 저축 금액과 쿠션 조건을 사용한다.
 처리·저장: BudgetEngine이 원화 정수로 배분하고 내부 예산 버전과 사용한 프로필 버전을 저장한다. 생활비 예산과 여윳돈의 경계를 구분해 같은 금액을 두 항목에 배치하지 않는다. 대출 상환은 대출의 월 상환 예정액으로 한 번만 넣고, 같은 상환 출금을 고정지출로 다시 넣지 않는다(TXN-008).
 예외: 필수 비용만으로 수입을 초과하면 부족액과 INFEASIBLE을 반환하고 저축이나 생활비를 임의 음수로 만들지 않는다.
 검수: 배분 합계는 수입 이하이고 잔여액의 위치가 설명되며, 하한과 1원 차이 및 수입 0원의 경우에도 합계가 보존된다.
@@ -1493,7 +1497,7 @@
         <is>
           <t>입력: 확정 예산 버전의 카테고리별 생활비 예산·사용액, 여윳돈, 선택 계좌의 최신 잔액과 미배정 확정 유입을 사용한다.
 처리·저장: 안전 소비액 = 남은 생활비 + 여윳돈. 고정지출·확정 카드대금·현재 회차 할부금·저축·쿠션은 각자의 예산으로 관리하므로 이 계산에서 다시 차감하지 않는다. 이미 잔액에 반영된 납부액·카드대금은 소비와 현금 유출을 중복 계산하지 않는다(COM-004).
-승인된 예산 기간 중에 고정지출이 새로 확정되면(TXN-008) 이번 주기 몫은 여윳돈에서 먼저 충당하고, 여윳돈이 모자라면 부족액만큼 예산 조정을 제안하며 사용자 승인 전에는 카테고리 예산을 바꾸지 않는다.
+승인된 예산 기간 중에 고정지출이 새로 확정되거나 금액이 바뀌거나 중지되면(TXN-008) 이번 주기 몫(또는 차액)은 여윳돈에서 먼저 충당하고(줄어든 금액은 여윳돈으로 돌림), 여윳돈이 모자라면 부족액만큼 예산 조정을 제안하며 사용자 승인 전에는 카테고리 예산을 바꾸지 않는다.
 예외: 미확정 수입·미수금은 여윳돈에 더하지 않고 미확정 비용은 확인 목록으로 표시한다. 남은 생활비가 음수(초과 사용)이면 0원으로 숨기지 않고 부족액으로 표시한다.
 검수: 남은 생활비 40만원·여윳돈 10만원이면 50만원이며, 고정지출 납부·카드대금 출금이 일어나도 안전 소비액이 이중 감소하지 않는다.
 참고 반영(OBL-001·002): 새 확정 정보는 현재 잔액·안전 소비액 재계산과 승인 예산 변경을 구분하고, 승인된 배분 자체를 조용히 덮어쓰지 않는다. 예상·미확인 항목은 출처·예정일·갱신 시각과 함께 별도 표시한다.</t>
@@ -4837,6 +4841,7 @@
       <c r="F122" s="17" t="inlineStr">
         <is>
           <t>검수 기준: 독립 기준 계산 대비 원 단위 금액 일치 100%, 보호 조건 위반·중복 차감·무승인 적용 0건을 품질 목표로 둔다.
+중복 방지(10/21 확정): 새로 만들기·승인 요청은 화면이 폼을 열 때 만든 요청 번호(Idempotency-Key)로 한 번만 반영하고(같은 번호 재요청은 처음 응답 반환), 저장 중에는 버튼을 잠근다. 이름이 같다는 이유로 중복이라고 판단하지 않는다.
 필수 사례: 카드 소비/결제, 내부이체, 부분 결제, 급여일·월 경계, 승인 직전 자료 변경, 동시 승인·중복 메시지, 타인 접근, 실패 후 재시도.
 예외: 미수집·미확인과 0원을 구별한다. 시험 표본·환경과 목표/실측 결과를 분리하고 미실행을 통과로 기록하지 않는다.
 추가 검수: 예산 조정 모드별 검수(합계 유지·초과 금액 전부 보충·이미 쓴 금액 아래 인하 금지·남은 생활비 범위), 자물쇠 유지, 재생성 3회 실패 전환, 복지·대출 동의 전 미실행, 미확정 지원금 예상 시나리오 표시, 월 상환금 한도 초과 상품 제외, 소비 분석 LLM 미사용, 잔소리 문구 표시 조건(조정 3회째·자물쇠 변경 3회)을 포함한다.</t>
@@ -5012,7 +5017,7 @@
       </c>
       <c r="F126" s="11" t="inlineStr">
         <is>
-          <t>입력: obligation_id, due_date, account_ref, confirmed_amount, paid_amount, status, 관련 거래 ID. 이미 잔액에 반영된 출금은 남은 의무지출에서 해소한다.
+          <t>입력: obligation_id, due_date, account_ref, confirmed_amount, paid_amount, status, 관련 거래 ID. 이미 잔액에 반영된 출금은 남은 의무지출에서 해소한다. 결제 수단별 기준(10/21 확정): 돈이 실제로 빠져나가는 길은 하나로만 센다. 계좌로 내는 고정지출은 그 고정지출이 납부 의무가 되고, 카드로 내는 고정지출은 따로 납부 의무를 만들지 않고 카드 청구서 안에 포함된 것으로 본다(예: 청구서 50만 원 안의 구독료 1만 원 → 나갈 돈은 50만 원 하나). 결제 수단을 모르는 고정지출은 일단 따로 세고, 카드 내역에서 발견되면 결제 수단을 카드로 바꿀지 묻는다. 대출 상환은 대출의 납부 의무 하나로만 센다. 예산(무엇을 썼나)과 꼭 나갈 돈(통장에서 언제 얼마가 빠지나)은 따로 계산하며, 카드로 낸 고정지출은 긁은 날 생활비 대신 고정비로 센다.
 검수 기준: 카드·부분결제·내부이체 사례에서 소비와 현금의 중복 반영 0건.</t>
         </is>
       </c>
@@ -5026,7 +5031,7 @@
           <t>공통 계산 기준
 TXN-003~009
 BUD-005
-CAL-005~009</t>
+CAL-005~009 / 10/21 수정</t>
         </is>
       </c>
     </row>

</xml_diff>